<commit_message>
Résolution jour 3 de nos exercices de préparation pour stage
</commit_message>
<xml_diff>
--- a/Analyses Excel/Préparation_Stage_Academique_2026_(exercices_pratique).xlsx
+++ b/Analyses Excel/Préparation_Stage_Academique_2026_(exercices_pratique).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JevainBkg\Projets\Datascience-roadmap\Analyses Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8543D832-3090-4FF4-9DFD-79B738AAB22B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D179E2-7A7C-4F37-8C8F-FD0F3115AF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="1" xr2:uid="{7D3A7277-DCDC-4547-AB5A-331124B03413}"/>
   </bookViews>
@@ -82,8 +82,30 @@
 </connections>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="194">
   <si>
     <t>transaction_id</t>
   </si>
@@ -708,12 +730,15 @@
   <si>
     <t>Segmentation des clients</t>
   </si>
+  <si>
+    <t xml:space="preserve">Canal fav </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -766,8 +791,15 @@
       <name val="Aptos Display"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -840,26 +872,8 @@
         <bgColor theme="9" tint="0.39997558519241921"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -890,6 +904,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -908,7 +931,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -964,7 +987,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1023,20 +1045,206 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="555">
+  <dxfs count="172">
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1128,73 +1336,63 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="0"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="-0.249977111117893"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="5"/>
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="5"/>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="5"/>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="5" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1207,1931 +1405,10 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
@@ -3473,20 +1750,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -3695,7 +1958,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>730249</xdr:colOff>
+      <xdr:colOff>698499</xdr:colOff>
       <xdr:row>83</xdr:row>
       <xdr:rowOff>179917</xdr:rowOff>
     </xdr:to>
@@ -3735,7 +1998,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="476250" y="19547417"/>
+              <a:off x="476250" y="18796000"/>
               <a:ext cx="6117166" cy="941917"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -4825,7 +3088,7 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="550">
+    <format dxfId="167">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -4834,7 +3097,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="549">
+    <format dxfId="166">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -4843,7 +3106,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="548">
+    <format dxfId="165">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -4852,7 +3115,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="547">
+    <format dxfId="164">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -4861,7 +3124,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="546">
+    <format dxfId="163">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -4870,7 +3133,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="545">
+    <format dxfId="162">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -4981,10 +3244,10 @@
     <dataField name="Somme de montant_fc" fld="6" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="507">
+    <format dxfId="126">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="506">
+    <format dxfId="125">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -5107,10 +3370,10 @@
     <dataField name="Somme de montant_fc" fld="6" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="5">
-    <format dxfId="512">
+    <format dxfId="131">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="511">
+    <format dxfId="130">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -5120,7 +3383,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="510">
+    <format dxfId="129">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="2">
@@ -5130,7 +3393,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="509">
+    <format dxfId="128">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="2">
@@ -5140,7 +3403,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="508">
+    <format dxfId="127">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="2">
@@ -5322,10 +3585,10 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="492">
+    <format dxfId="111">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="491">
+    <format dxfId="110">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -5406,13 +3669,13 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="495">
+    <format dxfId="114">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="494">
+    <format dxfId="113">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="493">
+    <format dxfId="112">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="1">
@@ -5503,10 +3766,10 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="497">
+    <format dxfId="116">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="496">
+    <format dxfId="115">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -5649,10 +3912,10 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="499">
+    <format dxfId="118">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="498">
+    <format dxfId="117">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -5737,10 +4000,10 @@
     <dataField name="CA" fld="5" baseField="6" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="446">
+    <format dxfId="65">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="445">
+    <format dxfId="64">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -5875,7 +4138,7 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="454">
+    <format dxfId="73">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -5887,7 +4150,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="453">
+    <format dxfId="72">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -5899,7 +4162,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="452">
+    <format dxfId="71">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -5911,7 +4174,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="451">
+    <format dxfId="70">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -5923,20 +4186,20 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="450">
+    <format dxfId="69">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="449">
+    <format dxfId="68">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="448">
+    <format dxfId="67">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="447">
+    <format dxfId="66">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -6049,7 +4312,7 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="460">
+    <format dxfId="79">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="4" selected="0">
@@ -6064,7 +4327,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="459">
+    <format dxfId="78">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="1" selected="0">
@@ -6076,7 +4339,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="458">
+    <format dxfId="77">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="1" selected="0">
@@ -6088,13 +4351,13 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="457">
+    <format dxfId="76">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="456">
+    <format dxfId="75">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="455">
+    <format dxfId="74">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -6271,29 +4534,29 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="24">
-    <format dxfId="484">
+    <format dxfId="103">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="483">
+    <format dxfId="102">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="482">
+    <format dxfId="101">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="481">
+    <format dxfId="100">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="480">
+    <format dxfId="99">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="479">
+    <format dxfId="98">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="478">
+    <format dxfId="97">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6306,7 +4569,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="477">
+    <format dxfId="96">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6319,7 +4582,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="476">
+    <format dxfId="95">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6332,7 +4595,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="475">
+    <format dxfId="94">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6345,7 +4608,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="474">
+    <format dxfId="93">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6358,7 +4621,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="473">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6371,7 +4634,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="472">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6384,7 +4647,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="471">
+    <format dxfId="90">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6397,7 +4660,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="470">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -6410,7 +4673,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="469">
+    <format dxfId="88">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1">
@@ -6422,7 +4685,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="468">
+    <format dxfId="87">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -6431,7 +4694,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="467">
+    <format dxfId="86">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -6440,7 +4703,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="466">
+    <format dxfId="85">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="7">
@@ -6455,7 +4718,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="465">
+    <format dxfId="84">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -6464,7 +4727,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="464">
+    <format dxfId="83">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -6473,7 +4736,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="463">
+    <format dxfId="82">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -6486,7 +4749,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="462">
+    <format dxfId="81">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -6499,7 +4762,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="461">
+    <format dxfId="80">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -6659,7 +4922,7 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="552">
+    <format dxfId="169">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -6668,7 +4931,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="551">
+    <format dxfId="168">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -6746,7 +5009,7 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="554">
+    <format dxfId="171">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="1">
@@ -6755,7 +5018,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="553">
+    <format dxfId="170">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="1">
@@ -6885,10 +5148,10 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="367">
+    <format dxfId="54">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="368">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -7010,7 +5273,7 @@
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{307774D1-06E3-4866-B6C8-A311F7479B8C}" name="Tableau croisé dynamique25" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B71:L77" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
+  <location ref="B71:F77" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisRow" numFmtId="14" showAll="0">
@@ -7024,9 +5287,9 @@
     <pivotField axis="axisCol" showAll="0">
       <items count="9">
         <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
+        <item h="1" x="1"/>
+        <item h="1" x="2"/>
+        <item h="1" x="3"/>
         <item h="1" x="4"/>
         <item h="1" x="5"/>
         <item h="1" x="6"/>
@@ -7068,30 +5331,9 @@
     <field x="2"/>
     <field x="-2"/>
   </colFields>
-  <colItems count="10">
+  <colItems count="4">
     <i>
       <x/>
-      <x/>
-    </i>
-    <i r="1" i="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x/>
-    </i>
-    <i r="1" i="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x/>
-    </i>
-    <i r="1" i="1">
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="3"/>
       <x/>
     </i>
     <i r="1" i="1">
@@ -7108,8 +5350,8 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="25">
-    <format dxfId="535">
+  <formats count="28">
+    <format dxfId="152">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="1" count="2">
@@ -7122,10 +5364,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="534">
+    <format dxfId="151">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="533">
+    <format dxfId="150">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7138,7 +5380,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="532">
+    <format dxfId="149">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7151,7 +5393,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="531">
+    <format dxfId="148">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7164,7 +5406,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="530">
+    <format dxfId="147">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7177,7 +5419,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="529">
+    <format dxfId="146">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7190,7 +5432,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="528">
+    <format dxfId="145">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7203,7 +5445,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="527">
+    <format dxfId="144">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7216,7 +5458,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="526">
+    <format dxfId="143">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -7229,7 +5471,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="525">
+    <format dxfId="142">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7238,7 +5480,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="524">
+    <format dxfId="141">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -7247,10 +5489,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="523">
+    <format dxfId="140">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="522">
+    <format dxfId="139">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="2" selected="0">
@@ -7267,7 +5509,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="521">
+    <format dxfId="138">
       <pivotArea dataOnly="0" labelOnly="1" offset="A256" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -7276,7 +5518,113 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="520">
+    <format dxfId="53">
+      <pivotArea dataOnly="0" labelOnly="1" offset="IV256" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="52">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="51">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="50">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="49">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="48">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="5"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="47">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="6"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="46">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="1">
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="33">
+      <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" axis="axisCol" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="2" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="32">
+      <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" axis="axisCol" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="31">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="2" selected="0">
+            <x v="0"/>
+            <x v="1"/>
+          </reference>
+          <reference field="1" count="1">
+            <x v="1"/>
+          </reference>
+          <reference field="2" count="0" selected="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="28">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -7285,13 +5633,11 @@
           <reference field="1" count="1">
             <x v="1"/>
           </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="0"/>
-          </reference>
+          <reference field="2" count="0" selected="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="519">
+    <format dxfId="0">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -7300,81 +5646,7 @@
           <reference field="1" count="1">
             <x v="1"/>
           </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="352">
-      <pivotArea dataOnly="0" labelOnly="1" offset="IV256" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="243">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="223">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="202">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="180">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="157">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="5"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="110">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="6"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="109">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="1">
-          <reference field="2" count="1">
-            <x v="7"/>
-          </reference>
+          <reference field="2" count="0" selected="0"/>
         </references>
       </pivotArea>
     </format>
@@ -7494,17 +5766,17 @@
     <dataField name="Canal preferé par client" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="364">
+    <format dxfId="43">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="365">
+    <format dxfId="44">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="366">
+    <format dxfId="45">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -7664,9 +5936,9 @@
     <tabular pivotCacheId="1733318224">
       <items count="8">
         <i x="0" s="1"/>
-        <i x="1" s="1"/>
-        <i x="2" s="1"/>
-        <i x="3" s="1"/>
+        <i x="1"/>
+        <i x="2"/>
+        <i x="3"/>
         <i x="4"/>
         <i x="5"/>
         <i x="6"/>
@@ -7684,16 +5956,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6EC83A65-D9A6-475F-8D16-1CE811FFF2E9}" name="Tableau1" displayName="Tableau1" ref="B3:H13" totalsRowShown="0" headerRowDxfId="544" dataDxfId="543">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6EC83A65-D9A6-475F-8D16-1CE811FFF2E9}" name="Tableau1" displayName="Tableau1" ref="B3:H13" totalsRowShown="0" headerRowDxfId="161" dataDxfId="160">
   <autoFilter ref="B3:H13" xr:uid="{6EC83A65-D9A6-475F-8D16-1CE811FFF2E9}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{54537CD7-847D-4C04-9BD6-B993FB8C0924}" name="transaction_id" dataDxfId="542"/>
-    <tableColumn id="2" xr3:uid="{7DFAA592-DC98-463C-A6AF-A94A0F915646}" name="date" dataDxfId="541"/>
-    <tableColumn id="3" xr3:uid="{122DF7BD-714F-4B55-830F-7573F364E80A}" name="client_id" dataDxfId="540"/>
-    <tableColumn id="4" xr3:uid="{1B94713D-DD23-416E-B23B-98EF629AFCBE}" name="commune" dataDxfId="539"/>
-    <tableColumn id="5" xr3:uid="{084E48D7-3EDD-4FC4-B38B-BD3872EDFF23}" name="produit" dataDxfId="538"/>
-    <tableColumn id="6" xr3:uid="{D1BF92F6-B520-4D49-B97E-C1395DDE5A98}" name="montant_fc" dataDxfId="537"/>
-    <tableColumn id="7" xr3:uid="{21C18558-D71D-47B7-B0D0-001594508953}" name="canal" dataDxfId="536"/>
+    <tableColumn id="1" xr3:uid="{54537CD7-847D-4C04-9BD6-B993FB8C0924}" name="transaction_id" dataDxfId="159"/>
+    <tableColumn id="2" xr3:uid="{7DFAA592-DC98-463C-A6AF-A94A0F915646}" name="date" dataDxfId="158"/>
+    <tableColumn id="3" xr3:uid="{122DF7BD-714F-4B55-830F-7573F364E80A}" name="client_id" dataDxfId="157"/>
+    <tableColumn id="4" xr3:uid="{1B94713D-DD23-416E-B23B-98EF629AFCBE}" name="commune" dataDxfId="156"/>
+    <tableColumn id="5" xr3:uid="{084E48D7-3EDD-4FC4-B38B-BD3872EDFF23}" name="produit" dataDxfId="155"/>
+    <tableColumn id="6" xr3:uid="{D1BF92F6-B520-4D49-B97E-C1395DDE5A98}" name="montant_fc" dataDxfId="154"/>
+    <tableColumn id="7" xr3:uid="{21C18558-D71D-47B7-B0D0-001594508953}" name="canal" dataDxfId="153"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7703,13 +5975,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5B43BC6D-66A6-432F-982F-C406FA282078}" name="Dataset_day2__2" displayName="Dataset_day2__2" ref="B2:H17" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="B2:H17" xr:uid="{5B43BC6D-66A6-432F-982F-C406FA282078}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F0363F15-00D8-44D9-B9E8-73E1201A36E6}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="518"/>
-    <tableColumn id="2" xr3:uid="{85F76B94-3323-41EB-B99E-F9DE7DD9EF5D}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="517"/>
-    <tableColumn id="3" xr3:uid="{90258075-E8BA-4181-AEBF-14DCE9CF1AC4}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="516"/>
-    <tableColumn id="4" xr3:uid="{3B088930-C813-470C-9790-11DA318C42A1}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="515"/>
-    <tableColumn id="5" xr3:uid="{E074DF00-E0E7-41D6-B91A-ABE22CB1881A}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="514"/>
+    <tableColumn id="1" xr3:uid="{F0363F15-00D8-44D9-B9E8-73E1201A36E6}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="137"/>
+    <tableColumn id="2" xr3:uid="{85F76B94-3323-41EB-B99E-F9DE7DD9EF5D}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="136"/>
+    <tableColumn id="3" xr3:uid="{90258075-E8BA-4181-AEBF-14DCE9CF1AC4}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="135"/>
+    <tableColumn id="4" xr3:uid="{3B088930-C813-470C-9790-11DA318C42A1}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="134"/>
+    <tableColumn id="5" xr3:uid="{E074DF00-E0E7-41D6-B91A-ABE22CB1881A}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="133"/>
     <tableColumn id="6" xr3:uid="{7C01ABE9-F9C0-40F6-9F95-D610FB820086}" uniqueName="6" name="montant_fc" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{30F6D1BA-4065-4D54-BF94-1BE05C99AC63}" uniqueName="7" name="canal" queryTableFieldId="7" dataDxfId="513"/>
+    <tableColumn id="7" xr3:uid="{30F6D1BA-4065-4D54-BF94-1BE05C99AC63}" uniqueName="7" name="canal" queryTableFieldId="7" dataDxfId="132"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7719,12 +5991,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A4A0DCA2-C1C4-44D4-AD45-BDA248A44995}" name="Dataset_day3" displayName="Dataset_day3" ref="B2:H17" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="B2:H17" xr:uid="{A4A0DCA2-C1C4-44D4-AD45-BDA248A44995}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A0067E32-0369-4D8A-BDF1-C8B907B86BD0}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="505"/>
-    <tableColumn id="2" xr3:uid="{C68FAFFA-BEA0-4F94-BA99-6450F477971E}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="504"/>
-    <tableColumn id="3" xr3:uid="{CDF65428-BE02-471D-A8F7-90F1D8454251}" uniqueName="3" name="agent_id" queryTableFieldId="3" dataDxfId="503"/>
-    <tableColumn id="4" xr3:uid="{22F84FAA-57F1-425F-B37C-F8428C49E033}" uniqueName="4" name="client_id" queryTableFieldId="4" dataDxfId="502"/>
-    <tableColumn id="5" xr3:uid="{93A8CFD1-D585-478D-9AFB-02301838500E}" uniqueName="5" name="commune" queryTableFieldId="5" dataDxfId="501"/>
-    <tableColumn id="6" xr3:uid="{956E7CEA-E833-4F96-9E51-2D67194B8C61}" uniqueName="6" name="produit" queryTableFieldId="6" dataDxfId="500"/>
+    <tableColumn id="1" xr3:uid="{A0067E32-0369-4D8A-BDF1-C8B907B86BD0}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{C68FAFFA-BEA0-4F94-BA99-6450F477971E}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="123"/>
+    <tableColumn id="3" xr3:uid="{CDF65428-BE02-471D-A8F7-90F1D8454251}" uniqueName="3" name="agent_id" queryTableFieldId="3" dataDxfId="122"/>
+    <tableColumn id="4" xr3:uid="{22F84FAA-57F1-425F-B37C-F8428C49E033}" uniqueName="4" name="client_id" queryTableFieldId="4" dataDxfId="121"/>
+    <tableColumn id="5" xr3:uid="{93A8CFD1-D585-478D-9AFB-02301838500E}" uniqueName="5" name="commune" queryTableFieldId="5" dataDxfId="120"/>
+    <tableColumn id="6" xr3:uid="{956E7CEA-E833-4F96-9E51-2D67194B8C61}" uniqueName="6" name="produit" queryTableFieldId="6" dataDxfId="119"/>
     <tableColumn id="7" xr3:uid="{E636C8A0-3C3C-48BE-AFE5-1B3DB129CA7E}" uniqueName="7" name="montant_fc" queryTableFieldId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -7735,11 +6007,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AB24B926-8F3E-4EE6-9138-D47BB2378B02}" name="Dataset_day4" displayName="Dataset_day4" ref="B2:G17" totalsRowShown="0">
   <autoFilter ref="B2:G17" xr:uid="{AB24B926-8F3E-4EE6-9138-D47BB2378B02}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{2FA77349-5B7D-430C-A299-CA8EF8B94F8F}" name="transaction_id" dataDxfId="490"/>
-    <tableColumn id="2" xr3:uid="{EA88A0A8-EDC4-468E-80F4-EF0578FE9A03}" name="date" dataDxfId="489"/>
-    <tableColumn id="3" xr3:uid="{811F8411-B146-492E-A697-2D905854F94D}" name="client_id" dataDxfId="488"/>
-    <tableColumn id="4" xr3:uid="{7B37CE19-01A8-4470-8A2B-849B751FB37D}" name="commune" dataDxfId="487"/>
-    <tableColumn id="5" xr3:uid="{863A1A63-AC11-4715-82E2-F6EC444E5B51}" name="produit" dataDxfId="486"/>
+    <tableColumn id="1" xr3:uid="{2FA77349-5B7D-430C-A299-CA8EF8B94F8F}" name="transaction_id" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{EA88A0A8-EDC4-468E-80F4-EF0578FE9A03}" name="date" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{811F8411-B146-492E-A697-2D905854F94D}" name="client_id" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{7B37CE19-01A8-4470-8A2B-849B751FB37D}" name="commune" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{863A1A63-AC11-4715-82E2-F6EC444E5B51}" name="produit" dataDxfId="105"/>
     <tableColumn id="6" xr3:uid="{DDFB738A-4C05-4F97-882D-16FE65EF8A7E}" name="montant_fc"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -7747,7 +6019,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B1C5B688-9C67-4CAD-9DAE-7207D5E5E850}" name="Tableau9" displayName="Tableau9" ref="AA3:AA11" totalsRowShown="0" headerRowDxfId="485">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B1C5B688-9C67-4CAD-9DAE-7207D5E5E850}" name="Tableau9" displayName="Tableau9" ref="AA3:AA11" totalsRowShown="0" headerRowDxfId="104">
   <autoFilter ref="AA3:AA11" xr:uid="{B1C5B688-9C67-4CAD-9DAE-7207D5E5E850}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="AA4:AA11">
     <sortCondition ref="AA3:AA11"/>
@@ -7762,16 +6034,16 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C4A92EC0-501A-4751-9A16-2163E0BD39EA}" name="Dataset_day5" displayName="Dataset_day5" ref="B2:H17" tableType="queryTable" totalsRowShown="0" headerRowDxfId="444">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C4A92EC0-501A-4751-9A16-2163E0BD39EA}" name="Dataset_day5" displayName="Dataset_day5" ref="B2:H17" tableType="queryTable" totalsRowShown="0" headerRowDxfId="63">
   <autoFilter ref="B2:H17" xr:uid="{C4A92EC0-501A-4751-9A16-2163E0BD39EA}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{FBC21564-1B48-423F-AFDB-04B5AE20CF75}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="443"/>
-    <tableColumn id="2" xr3:uid="{CA4A50D7-5720-4F71-ACD1-3781681C0231}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="442"/>
-    <tableColumn id="3" xr3:uid="{A265E5F8-50A6-4DD3-8C5E-10BB05E3F126}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="441"/>
-    <tableColumn id="4" xr3:uid="{0E595B89-2727-474B-B4A6-66BC0AC0864A}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="440"/>
-    <tableColumn id="5" xr3:uid="{4D992877-9744-466D-982E-E1F06CDEF762}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="439"/>
+    <tableColumn id="1" xr3:uid="{FBC21564-1B48-423F-AFDB-04B5AE20CF75}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{CA4A50D7-5720-4F71-ACD1-3781681C0231}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{A265E5F8-50A6-4DD3-8C5E-10BB05E3F126}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="60"/>
+    <tableColumn id="4" xr3:uid="{0E595B89-2727-474B-B4A6-66BC0AC0864A}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{4D992877-9744-466D-982E-E1F06CDEF762}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="58"/>
     <tableColumn id="6" xr3:uid="{D10FAE6E-7969-4551-94AB-82C2D27DFD50}" uniqueName="6" name="montant_fc" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{7306D68B-3C9A-40F7-A0D9-E00CC8C73541}" uniqueName="7" name="periode" queryTableFieldId="7" dataDxfId="438"/>
+    <tableColumn id="7" xr3:uid="{7306D68B-3C9A-40F7-A0D9-E00CC8C73541}" uniqueName="7" name="periode" queryTableFieldId="7" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7782,7 +6054,7 @@
   <autoFilter ref="A1:G6" xr:uid="{68E59C74-D329-4B48-A967-CC868365949C}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C102BD58-3DF8-48B7-9114-2067608D3DB4}" name="transaction_id"/>
-    <tableColumn id="2" xr3:uid="{998F6E83-476D-414D-8353-8E6146354739}" name="date" dataDxfId="437"/>
+    <tableColumn id="2" xr3:uid="{998F6E83-476D-414D-8353-8E6146354739}" name="date" dataDxfId="56"/>
     <tableColumn id="3" xr3:uid="{1ACC5CD9-2A0F-4DB2-B7B7-A25781DA1795}" name="agent_id"/>
     <tableColumn id="4" xr3:uid="{D4B111D2-01DE-4AFC-91B0-641E23172B8C}" name="client_id"/>
     <tableColumn id="5" xr3:uid="{C0E2906A-2633-4FB3-89D8-883ADDF86D4F}" name="commune"/>
@@ -8121,15 +6393,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="47" t="s">
+      <c r="B2" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
@@ -8428,18 +6700,18 @@
       <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="44" t="s">
+      <c r="B15" s="43" t="s">
         <v>171</v>
       </c>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="48"/>
     </row>
     <row r="16" spans="1:9" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="37"/>
+      <c r="B16" s="36"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -8448,18 +6720,18 @@
       <c r="H16" s="1"/>
     </row>
     <row r="17" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="43" t="s">
         <v>172</v>
       </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="38"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="37"/>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="47"/>
+      <c r="C19" s="46"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
@@ -8506,20 +6778,20 @@
       <c r="C26" s="10"/>
     </row>
     <row r="27" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="44" t="s">
+      <c r="B27" s="43" t="s">
         <v>173</v>
       </c>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="38"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="37"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="47" t="s">
+      <c r="B30" s="46" t="s">
         <v>45</v>
       </c>
-      <c r="C30" s="47"/>
+      <c r="C30" s="46"/>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
@@ -8530,7 +6802,7 @@
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="39" t="s">
+      <c r="B32" s="38" t="s">
         <v>9</v>
       </c>
       <c r="C32" s="21">
@@ -8578,17 +6850,17 @@
       </c>
     </row>
     <row r="40" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B40" s="44" t="s">
+      <c r="B40" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="C40" s="44"/>
-      <c r="D40" s="44"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B42" s="47" t="s">
+      <c r="B42" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="C42" s="47"/>
+      <c r="C42" s="46"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
@@ -8639,17 +6911,17 @@
       </c>
     </row>
     <row r="50" spans="2:5" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B50" s="44" t="s">
+      <c r="B50" s="43" t="s">
         <v>175</v>
       </c>
-      <c r="C50" s="44"/>
-      <c r="D50" s="44"/>
+      <c r="C50" s="43"/>
+      <c r="D50" s="43"/>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B52" s="47" t="s">
+      <c r="B52" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="C52" s="48"/>
+      <c r="C52" s="47"/>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" s="8" t="s">
@@ -8692,56 +6964,56 @@
       </c>
     </row>
     <row r="60" spans="2:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B60" s="45" t="s">
+      <c r="B60" s="44" t="s">
         <v>182</v>
       </c>
-      <c r="C60" s="45"/>
+      <c r="C60" s="44"/>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B62" s="46" t="s">
+      <c r="B62" s="45" t="s">
         <v>183</v>
       </c>
-      <c r="C62" s="46"/>
-      <c r="D62" s="46"/>
-      <c r="E62" s="46"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
+      <c r="E62" s="45"/>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B63" s="46"/>
-      <c r="C63" s="46"/>
-      <c r="D63" s="46"/>
-      <c r="E63" s="46"/>
+      <c r="B63" s="45"/>
+      <c r="C63" s="45"/>
+      <c r="D63" s="45"/>
+      <c r="E63" s="45"/>
     </row>
     <row r="64" spans="2:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B64" s="41"/>
-      <c r="C64" s="41"/>
-      <c r="D64" s="41"/>
-      <c r="E64" s="41"/>
+      <c r="B64" s="40"/>
+      <c r="C64" s="40"/>
+      <c r="D64" s="40"/>
+      <c r="E64" s="40"/>
     </row>
     <row r="65" spans="2:2" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B65" s="42" t="s">
+      <c r="B65" s="41" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" s="40"/>
+      <c r="B66" s="39"/>
     </row>
     <row r="67" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B67" s="43" t="s">
+      <c r="B67" s="42" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="68" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B68" s="43" t="s">
+      <c r="B68" s="42" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="69" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B69" s="43" t="s">
+      <c r="B69" s="42" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="70" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B70" s="43" t="s">
+      <c r="B70" s="42" t="s">
         <v>181</v>
       </c>
     </row>
@@ -8813,9 +7085,9 @@
     <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.140625" customWidth="1"/>
@@ -9200,47 +7472,47 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="44" t="s">
+      <c r="B19" s="43" t="s">
         <v>171</v>
       </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="48"/>
     </row>
     <row r="20" spans="2:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="37"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
     </row>
     <row r="21" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="44" t="s">
+      <c r="B21" s="43" t="s">
         <v>184</v>
       </c>
-      <c r="C21" s="44"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="44"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
     </row>
     <row r="22" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
     </row>
     <row r="23" spans="2:8" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B23" s="44" t="s">
+      <c r="B23" s="43" t="s">
         <v>185</v>
       </c>
-      <c r="C23" s="44"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="38"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
     </row>
     <row r="24" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
@@ -9331,26 +7603,26 @@
       <c r="C35" s="10"/>
     </row>
     <row r="36" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="44" t="s">
+      <c r="B36" s="43" t="s">
         <v>186</v>
       </c>
-      <c r="C36" s="44"/>
-      <c r="D36" s="44"/>
-      <c r="E36" s="44"/>
+      <c r="C36" s="43"/>
+      <c r="D36" s="43"/>
+      <c r="E36" s="43"/>
     </row>
     <row r="37" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="37"/>
-      <c r="C37" s="37"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="37"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="36"/>
+      <c r="D37" s="36"/>
+      <c r="E37" s="36"/>
     </row>
     <row r="38" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="44" t="s">
+      <c r="B38" s="43" t="s">
         <v>189</v>
       </c>
-      <c r="C38" s="44"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="37"/>
+      <c r="C38" s="43"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="36"/>
     </row>
     <row r="39" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="18" t="s">
@@ -9432,39 +7704,40 @@
         <v>167000</v>
       </c>
     </row>
-    <row r="49" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="44" t="s">
+    <row r="49" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="43" t="s">
         <v>188</v>
       </c>
-      <c r="C51" s="44"/>
-      <c r="D51" s="44"/>
-      <c r="E51" s="44"/>
-    </row>
-    <row r="52" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="37"/>
-      <c r="C52" s="37"/>
-      <c r="D52" s="37"/>
-      <c r="E52" s="37"/>
-    </row>
-    <row r="53" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B53" s="37" t="s">
+      <c r="C51" s="43"/>
+      <c r="D51" s="43"/>
+      <c r="E51" s="43"/>
+    </row>
+    <row r="52" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="36"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="36"/>
+      <c r="E52" s="36"/>
+    </row>
+    <row r="53" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="36" t="s">
         <v>187</v>
       </c>
-      <c r="C53" s="37"/>
-      <c r="D53" s="37"/>
-      <c r="E53" s="37"/>
-    </row>
-    <row r="54" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="36"/>
+      <c r="D53" s="36"/>
+      <c r="E53" s="36"/>
+    </row>
+    <row r="54" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="8" t="s">
         <v>72</v>
       </c>
       <c r="C54" s="8" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="55" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G54" s="49"/>
+    </row>
+    <row r="55" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B55" s="18" t="s">
         <v>74</v>
       </c>
@@ -9480,8 +7753,11 @@
       <c r="F55" s="11" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="56" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G55" s="52" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="9" t="s">
         <v>8</v>
       </c>
@@ -9493,8 +7769,12 @@
       <c r="F56" s="10">
         <v>7</v>
       </c>
-    </row>
-    <row r="57" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G56" s="10" t="str" cm="1">
+        <f t="array" ref="G56">_xlfn.IFS(MAX(C56:E56)=C56,"Agent",MAX(C56:E56)=D56,"Mobile Money",MAX(C56:E56)=E56,"USSD")</f>
+        <v>Mobile Money</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B57" s="9" t="s">
         <v>13</v>
       </c>
@@ -9506,8 +7786,12 @@
       <c r="F57" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="58" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G57" s="10" t="str" cm="1">
+        <f t="array" ref="G57">_xlfn.IFS(MAX(C57:E57)=C57,"Agent",MAX(C57:E57)=D57,"Mobile Money",MAX(C57:E57)=E57,"USSD")</f>
+        <v>USSD</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="9" t="s">
         <v>52</v>
       </c>
@@ -9519,8 +7803,12 @@
       <c r="F58" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G58" s="10" t="str" cm="1">
+        <f t="array" ref="G58">_xlfn.IFS(MAX(C58:E58)=C58,"Agent",MAX(C58:E58)=D58,"Mobile Money",MAX(C58:E58)=E58,"USSD")</f>
+        <v>Agent</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="9" t="s">
         <v>54</v>
       </c>
@@ -9532,8 +7820,12 @@
       <c r="F59" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G59" s="10" t="str" cm="1">
+        <f t="array" ref="G59">_xlfn.IFS(MAX(C59:E59)=C59,"Agent",MAX(C59:E59)=D59,"Mobile Money",MAX(C59:E59)=E59,"USSD")</f>
+        <v>Agent</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="9" t="s">
         <v>58</v>
       </c>
@@ -9545,8 +7837,12 @@
       <c r="F60" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G60" s="10" t="str" cm="1">
+        <f t="array" ref="G60">_xlfn.IFS(MAX(C60:E60)=C60,"Agent",MAX(C60:E60)=D60,"Mobile Money",MAX(C60:E60)=E60,"USSD")</f>
+        <v>Agent</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="9" t="s">
         <v>61</v>
       </c>
@@ -9558,8 +7854,12 @@
       <c r="F61" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G61" s="10" t="str" cm="1">
+        <f t="array" ref="G61">_xlfn.IFS(MAX(C61:E61)=C61,"Agent",MAX(C61:E61)=D61,"Mobile Money",MAX(C61:E61)=E61,"USSD")</f>
+        <v>Mobile Money</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="9" t="s">
         <v>64</v>
       </c>
@@ -9571,8 +7871,12 @@
       <c r="F62" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G62" s="10" t="str" cm="1">
+        <f t="array" ref="G62">_xlfn.IFS(MAX(C62:E62)=C62,"Agent",MAX(C62:E62)=D62,"Mobile Money",MAX(C62:E62)=E62,"USSD")</f>
+        <v>USSD</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B63" s="9" t="s">
         <v>67</v>
       </c>
@@ -9584,56 +7888,61 @@
       <c r="F63" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="64" spans="2:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G63" s="10" t="str" cm="1">
+        <f t="array" ref="G63">_xlfn.IFS(MAX(C63:E63)=C63,"Agent",MAX(C63:E63)=D63,"Mobile Money",MAX(C63:E63)=E63,"USSD")</f>
+        <v>Agent</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="9" t="s">
         <v>40</v>
       </c>
       <c r="C64" s="10">
         <v>4</v>
       </c>
-      <c r="E64" s="37"/>
-      <c r="F64" s="37"/>
+      <c r="E64" s="36"/>
+      <c r="F64" s="36"/>
+      <c r="G64" s="53"/>
     </row>
     <row r="65" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="37"/>
-      <c r="C65" s="37"/>
-      <c r="D65" s="37"/>
-      <c r="E65" s="37"/>
+      <c r="B65" s="36"/>
+      <c r="C65" s="36"/>
+      <c r="D65" s="36"/>
+      <c r="E65" s="36"/>
     </row>
     <row r="66" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="37"/>
-      <c r="C66" s="37"/>
-      <c r="D66" s="37"/>
-      <c r="E66" s="37"/>
+      <c r="B66" s="36"/>
+      <c r="C66" s="36"/>
+      <c r="D66" s="36"/>
+      <c r="E66" s="36"/>
     </row>
     <row r="67" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B67" s="44" t="s">
+      <c r="B67" s="43" t="s">
         <v>190</v>
       </c>
-      <c r="C67" s="44"/>
-      <c r="D67" s="44"/>
-      <c r="E67" s="44"/>
+      <c r="C67" s="43"/>
+      <c r="D67" s="43"/>
+      <c r="E67" s="43"/>
     </row>
     <row r="68" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B68" s="37"/>
-      <c r="C68" s="37"/>
-      <c r="D68" s="37"/>
-      <c r="E68" s="37"/>
+      <c r="B68" s="36"/>
+      <c r="C68" s="36"/>
+      <c r="D68" s="36"/>
+      <c r="E68" s="36"/>
     </row>
     <row r="69" spans="2:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B69" s="44" t="s">
+      <c r="B69" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="C69" s="44"/>
-      <c r="D69" s="44"/>
-      <c r="E69" s="44"/>
-      <c r="F69" s="44"/>
-      <c r="G69" s="44"/>
+      <c r="C69" s="43"/>
+      <c r="D69" s="43"/>
+      <c r="E69" s="43"/>
+      <c r="F69" s="43"/>
+      <c r="G69" s="43"/>
     </row>
     <row r="70" spans="2:20" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B70" s="44"/>
-      <c r="C70" s="44"/>
+      <c r="B70" s="43"/>
+      <c r="C70" s="43"/>
       <c r="F70" s="9"/>
       <c r="G70" s="10"/>
       <c r="H70" s="10"/>
@@ -9645,31 +7954,19 @@
         <v>42</v>
       </c>
     </row>
-    <row r="72" spans="2:20" ht="60" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:20" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C72" s="22" t="s">
         <v>8</v>
       </c>
       <c r="D72" s="22"/>
-      <c r="E72" s="50" t="s">
-        <v>13</v>
-      </c>
-      <c r="F72" s="50"/>
-      <c r="G72" s="51" t="s">
-        <v>52</v>
-      </c>
-      <c r="H72" s="51"/>
-      <c r="I72" s="52" t="s">
-        <v>54</v>
-      </c>
-      <c r="J72" s="52"/>
-      <c r="K72" s="19" t="s">
+      <c r="E72" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="L72" s="19" t="s">
+      <c r="F72" s="19" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="73" spans="2:20" s="19" customFormat="1" ht="90" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:20" s="19" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="B73" s="20" t="s">
         <v>38</v>
       </c>
@@ -9679,24 +7976,12 @@
       <c r="D73" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E73" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="F73" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="G73" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="H73" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="I73" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="J73" s="19" t="s">
-        <v>41</v>
-      </c>
+      <c r="G73"/>
+      <c r="H73"/>
+      <c r="I73"/>
+      <c r="J73"/>
+      <c r="K73"/>
+      <c r="L73"/>
       <c r="M73"/>
       <c r="N73"/>
       <c r="O73"/>
@@ -9717,55 +8002,27 @@
         <v>28000</v>
       </c>
       <c r="E74" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F74" s="10">
-        <v>3000</v>
-      </c>
-      <c r="G74" s="10">
-        <v>1</v>
-      </c>
-      <c r="H74" s="10">
-        <v>1000</v>
-      </c>
-      <c r="I74" s="10">
-        <v>1</v>
-      </c>
-      <c r="J74" s="10">
-        <v>18000</v>
-      </c>
-      <c r="K74" s="10">
-        <v>5</v>
-      </c>
-      <c r="L74" s="10">
-        <v>50000</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="75" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B75" s="17">
         <v>46147</v>
       </c>
-      <c r="C75" s="23">
+      <c r="C75" s="55">
         <v>4</v>
       </c>
-      <c r="D75" s="23">
+      <c r="D75" s="55">
         <v>64000</v>
       </c>
       <c r="E75" s="10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F75" s="10">
-        <v>3000</v>
-      </c>
-      <c r="G75" s="10"/>
-      <c r="H75" s="10"/>
-      <c r="I75" s="10"/>
-      <c r="J75" s="10"/>
-      <c r="K75" s="10">
-        <v>5</v>
-      </c>
-      <c r="L75" s="10">
-        <v>67000</v>
+        <v>64000</v>
       </c>
     </row>
     <row r="76" spans="2:20" x14ac:dyDescent="0.25">
@@ -9778,16 +8035,10 @@
       <c r="D76" s="10">
         <v>18000</v>
       </c>
-      <c r="E76" s="10"/>
-      <c r="F76" s="10"/>
-      <c r="G76" s="10"/>
-      <c r="H76" s="10"/>
-      <c r="I76" s="10"/>
-      <c r="J76" s="10"/>
-      <c r="K76" s="10">
+      <c r="E76" s="10">
         <v>1</v>
       </c>
-      <c r="L76" s="10">
+      <c r="F76" s="10">
         <v>18000</v>
       </c>
     </row>
@@ -9795,35 +8046,17 @@
       <c r="B77" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C77" s="10">
+      <c r="C77" s="54">
         <v>7</v>
       </c>
-      <c r="D77" s="10">
+      <c r="D77" s="54">
         <v>110000</v>
       </c>
       <c r="E77" s="10">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F77" s="10">
-        <v>6000</v>
-      </c>
-      <c r="G77" s="10">
-        <v>1</v>
-      </c>
-      <c r="H77" s="10">
-        <v>1000</v>
-      </c>
-      <c r="I77" s="10">
-        <v>1</v>
-      </c>
-      <c r="J77" s="10">
-        <v>18000</v>
-      </c>
-      <c r="K77" s="10">
-        <v>11</v>
-      </c>
-      <c r="L77" s="10">
-        <v>135000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="78" spans="2:20" x14ac:dyDescent="0.25">
@@ -9840,10 +8073,10 @@
       <c r="L78" s="10"/>
     </row>
     <row r="79" spans="2:20" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B79" s="53" t="s">
+      <c r="B79" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="C79" s="54"/>
+      <c r="C79" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9871,14 +8104,15 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <drawing r:id="rId6"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
       <x14:slicerList>
-        <x14:slicer r:id="rId7"/>
+        <x14:slicer r:id="rId8"/>
       </x14:slicerList>
     </ext>
   </extLst>
@@ -9925,16 +8159,16 @@
       <c r="H2" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="47" t="s">
+      <c r="J2" s="46" t="s">
         <v>111</v>
       </c>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="N2" s="47" t="s">
+      <c r="K2" s="46"/>
+      <c r="L2" s="46"/>
+      <c r="N2" s="46" t="s">
         <v>112</v>
       </c>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="2:16" ht="45" x14ac:dyDescent="0.25">
       <c r="B3" s="10" t="s">
@@ -10123,7 +8357,7 @@
       <c r="H7">
         <v>18000</v>
       </c>
-      <c r="J7" s="24" t="s">
+      <c r="J7" s="23" t="s">
         <v>80</v>
       </c>
       <c r="K7" s="10">
@@ -10164,7 +8398,7 @@
       <c r="H8">
         <v>18000</v>
       </c>
-      <c r="J8" s="24" t="s">
+      <c r="J8" s="23" t="s">
         <v>85</v>
       </c>
       <c r="K8" s="10">
@@ -10523,22 +8757,22 @@
     <mergeCell ref="N2:P2"/>
   </mergeCells>
   <conditionalFormatting pivot="1" sqref="L4:L8">
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="42" priority="5" operator="lessThan">
       <formula>10000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="P4:P8">
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="41" priority="4" operator="lessThan">
       <formula>$Q$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="P4:P9">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="3" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J7:J8">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="39" priority="1" operator="lessThan">
       <formula>10000</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10676,7 +8910,7 @@
       <c r="Y3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="AA3" s="27" t="s">
+      <c r="AA3" s="26" t="s">
         <v>136</v>
       </c>
     </row>
@@ -11278,7 +9512,7 @@
       <c r="H21" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="I21" s="25">
+      <c r="I21" s="24">
         <v>6</v>
       </c>
     </row>
@@ -11402,23 +9636,23 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B20:C29">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="38" priority="5" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="F21:F25">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="37" priority="4" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="F21:F25">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA4:AA11">
-    <cfRule type="top10" dxfId="1" priority="1" rank="2"/>
-    <cfRule type="top10" dxfId="0" priority="2" rank="2"/>
+    <cfRule type="top10" dxfId="35" priority="1" rank="2"/>
+    <cfRule type="top10" dxfId="34" priority="2" rank="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
@@ -11629,7 +9863,7 @@
       <c r="J5" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K5" s="30">
+      <c r="K5" s="29">
         <v>2</v>
       </c>
       <c r="L5" s="10">
@@ -11639,16 +9873,16 @@
         <v>1</v>
       </c>
       <c r="N5" s="10"/>
-      <c r="O5" s="25">
+      <c r="O5" s="24">
         <v>1</v>
       </c>
-      <c r="P5" s="25">
+      <c r="P5" s="24">
         <v>1</v>
       </c>
-      <c r="Q5" s="25">
+      <c r="Q5" s="24">
         <v>1</v>
       </c>
-      <c r="R5" s="25">
+      <c r="R5" s="24">
         <v>1</v>
       </c>
       <c r="S5" s="10"/>
@@ -11693,7 +9927,7 @@
       <c r="P6" s="10"/>
       <c r="Q6" s="10"/>
       <c r="R6" s="10"/>
-      <c r="S6" s="25">
+      <c r="S6" s="24">
         <v>1</v>
       </c>
       <c r="T6" s="10">
@@ -11778,22 +10012,22 @@
       <c r="H8" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="J8" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="K8" s="35" t="s">
+      <c r="K8" s="34" t="s">
         <v>147</v>
       </c>
-      <c r="L8" s="35" t="s">
+      <c r="L8" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="M8" s="35" t="s">
+      <c r="M8" s="34" t="s">
         <v>153</v>
       </c>
-      <c r="N8" s="35" t="s">
+      <c r="N8" s="34" t="s">
         <v>157</v>
       </c>
-      <c r="O8" s="35" t="s">
+      <c r="O8" s="34" t="s">
         <v>163</v>
       </c>
     </row>
@@ -11819,10 +10053,10 @@
       <c r="H9" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="J9" s="31" t="s">
+      <c r="J9" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="K9" s="31" t="s">
+      <c r="K9" s="30" t="s">
         <v>114</v>
       </c>
     </row>
@@ -11902,25 +10136,25 @@
       </c>
     </row>
     <row r="13" spans="2:20" s="19" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="31" t="s">
         <v>155</v>
       </c>
-      <c r="C13" s="33">
+      <c r="C13" s="32">
         <v>46159</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="E13" s="32" t="s">
+      <c r="E13" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="32" t="s">
+      <c r="F13" s="31" t="s">
         <v>10</v>
       </c>
       <c r="G13" s="19">
         <v>10000</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="H13" s="31" t="s">
         <v>144</v>
       </c>
       <c r="J13" s="20" t="s">
@@ -12028,26 +10262,26 @@
       <c r="J15" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="K15" s="25">
+      <c r="K15" s="24">
         <v>1</v>
       </c>
       <c r="L15" s="10">
         <v>2</v>
       </c>
-      <c r="M15" s="25">
+      <c r="M15" s="24">
         <v>1</v>
       </c>
       <c r="N15" s="10">
         <v>1</v>
       </c>
-      <c r="O15" s="25">
+      <c r="O15" s="24">
         <v>1</v>
       </c>
       <c r="P15" s="10">
         <v>1</v>
       </c>
       <c r="Q15" s="10"/>
-      <c r="R15" s="25">
+      <c r="R15" s="24">
         <v>1</v>
       </c>
       <c r="S15" s="10"/>
@@ -12092,7 +10326,7 @@
       <c r="P16" s="10"/>
       <c r="Q16" s="10"/>
       <c r="R16" s="10"/>
-      <c r="S16" s="25">
+      <c r="S16" s="24">
         <v>1</v>
       </c>
       <c r="T16" s="10">
@@ -12156,7 +10390,7 @@
       </c>
     </row>
     <row r="18" spans="2:38" x14ac:dyDescent="0.25">
-      <c r="J18" s="29" t="s">
+      <c r="J18" s="28" t="s">
         <v>167</v>
       </c>
     </row>
@@ -12185,42 +10419,42 @@
       <c r="AG19" s="19"/>
     </row>
     <row r="20" spans="2:38" s="19" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N20" s="34" t="s">
+      <c r="N20" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="O20" s="34"/>
-      <c r="P20" s="28" t="s">
+      <c r="O20" s="33"/>
+      <c r="P20" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="Q20" s="28"/>
-      <c r="R20" s="34" t="s">
+      <c r="Q20" s="27"/>
+      <c r="R20" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="S20" s="34"/>
-      <c r="T20" s="28" t="s">
+      <c r="S20" s="33"/>
+      <c r="T20" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="U20" s="28"/>
-      <c r="V20" s="34" t="s">
+      <c r="U20" s="27"/>
+      <c r="V20" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="W20" s="34"/>
-      <c r="X20" s="28" t="s">
+      <c r="W20" s="33"/>
+      <c r="X20" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="Y20" s="28"/>
-      <c r="Z20" s="34" t="s">
+      <c r="Y20" s="27"/>
+      <c r="Z20" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="AA20" s="34"/>
-      <c r="AB20" s="28" t="s">
+      <c r="AA20" s="33"/>
+      <c r="AB20" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="AC20" s="28"/>
-      <c r="AD20" s="34" t="s">
+      <c r="AC20" s="27"/>
+      <c r="AD20" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="AE20" s="34"/>
+      <c r="AE20" s="33"/>
       <c r="AF20" s="19" t="s">
         <v>70</v>
       </c>
@@ -12308,13 +10542,13 @@
       <c r="M22" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="N22" s="25">
+      <c r="N22" s="24">
         <v>18000</v>
       </c>
-      <c r="O22" s="25">
+      <c r="O22" s="24">
         <v>1</v>
       </c>
-      <c r="P22" s="25">
+      <c r="P22" s="24">
         <v>3000</v>
       </c>
       <c r="Q22" s="21">
@@ -12359,13 +10593,13 @@
       <c r="M23" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="N23" s="25">
+      <c r="N23" s="24">
         <v>25200</v>
       </c>
-      <c r="O23" s="25">
+      <c r="O23" s="24">
         <v>2</v>
       </c>
-      <c r="P23" s="25">
+      <c r="P23" s="24">
         <v>3000</v>
       </c>
       <c r="Q23" s="21">
@@ -12422,13 +10656,13 @@
       <c r="M24" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="N24" s="25">
+      <c r="N24" s="24">
         <v>18000</v>
       </c>
-      <c r="O24" s="25">
+      <c r="O24" s="24">
         <v>1</v>
       </c>
-      <c r="P24" s="25">
+      <c r="P24" s="24">
         <v>3000</v>
       </c>
       <c r="Q24" s="21">
@@ -12531,10 +10765,10 @@
       </c>
     </row>
     <row r="26" spans="2:38" x14ac:dyDescent="0.25">
-      <c r="J26" s="26" t="s">
+      <c r="J26" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="M26" s="29" t="s">
+      <c r="M26" s="28" t="s">
         <v>169</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update des Fichiers Jour4
</commit_message>
<xml_diff>
--- a/Analyses Excel/Préparation_Stage_Academique_2026_(exercices_pratique).xlsx
+++ b/Analyses Excel/Préparation_Stage_Academique_2026_(exercices_pratique).xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JevainBkg\Projets\Datascience-roadmap\Analyses Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8C1A734-BDA7-4378-8725-97A2C2A990CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BD14AF-B1A9-45BF-9624-ADE1DA15E3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13740" activeTab="3" xr2:uid="{7D3A7277-DCDC-4547-AB5A-331124B03413}"/>
   </bookViews>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="221">
   <si>
     <t>transaction_id</t>
   </si>
@@ -980,6 +980,95 @@
   </si>
   <si>
     <t>Classement agents</t>
+  </si>
+  <si>
+    <t>Question 1 : Quels clients semblent les plus fidèles ?</t>
+  </si>
+  <si>
+    <t>Fidelité  clients</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Note : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nos clients les plus fidèles sont c201, C202, C203; le reste de clients présente malheureusement un profil "one shot"</t>
+    </r>
+  </si>
+  <si>
+    <t>Question 2 : Quelle commune fidélise le mieux ?</t>
+  </si>
+  <si>
+    <t>Fidelisation commune</t>
+  </si>
+  <si>
+    <t>Pourcentage de fidélisation</t>
+  </si>
+  <si>
+    <t>Question 3 : Quel produit favorise le plus la récurrence ?</t>
+  </si>
+  <si>
+    <t>Fréquence produit</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Note : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>la majorité de nos clients opte pour le forfait mensuel Airbox de Data 10GB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Remarque  : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Alors, dans le souci d'améliorer notre taux de rétention ainsi que nos chiffres par la même occasion, je proposerai une campagne publicitaire bien ciblé, présentant nos autres offres tel que sms, Voice, leurs avantages ou utilités dans la vie courante, du cross-selling, ainsi qu'un petit sondage dans les zones masina, matete et ndjili histoire d'avoir un feedback du pourquoi le marché nous est capricieux dans ces dites zones Merci</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Note : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Nous noterons également le taux de fidélisation élevé de la zone Gombe</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1177,10 +1266,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1312,6 +1402,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1324,11 +1417,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="164">
+  <dxfs count="191">
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1341,11 +1472,13 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color theme="1"/>
       </font>
+    </dxf>
+    <dxf>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1371,11 +1504,23 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1391,11 +1536,13 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color theme="1"/>
       </font>
+    </dxf>
+    <dxf>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1411,11 +1558,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1460,108 +1617,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4DD36D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <fgColor theme="9" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF4DD36D"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -1580,6 +1635,271 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
@@ -1828,19 +2148,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
@@ -3348,7 +3655,7 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="155">
+    <format dxfId="182">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -3357,7 +3664,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="154">
+    <format dxfId="181">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="1">
@@ -3535,10 +3842,10 @@
     <dataField name="Somme de montant_fc" fld="6" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="105">
+    <format dxfId="132">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="104">
+    <format dxfId="131">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -3548,7 +3855,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="103">
+    <format dxfId="130">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="2">
@@ -3558,7 +3865,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="102">
+    <format dxfId="129">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="2">
@@ -3568,7 +3875,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="101">
+    <format dxfId="128">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="2">
@@ -3578,7 +3885,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="31">
+    <format dxfId="61">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
@@ -3775,10 +4082,10 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="87">
+    <format dxfId="117">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="86">
+    <format dxfId="116">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -3796,7 +4103,7 @@
 
 <file path=xl/pivotTables/pivotTable13.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6CF2CD07-335D-47F6-B7D4-64AD9F8422C1}" name="Tableau croisé dynamique34" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="H20:I25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="B56:C61" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField dataField="1" showAll="0">
       <items count="16">
@@ -3859,13 +4166,13 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="90">
+    <format dxfId="119">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="89">
+    <format dxfId="118">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="88">
+    <format dxfId="37">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="1">
@@ -3875,6 +4182,64 @@
       </pivotArea>
     </format>
   </formats>
+  <conditionalFormats count="4">
+    <conditionalFormat priority="12">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="4" count="1">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+    <conditionalFormat priority="11">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="4" count="1">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+    <conditionalFormat priority="10">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="4" count="1">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+    <conditionalFormat priority="9">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="4" count="1">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+  </conditionalFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -3889,7 +4254,7 @@
 
 <file path=xl/pivotTables/pivotTable14.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{12A32755-1450-4078-8441-200639987E8B}" name="Tableau croisé dynamique33" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E20:F26" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="B41:C47" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField dataField="1" showAll="0">
       <items count="16">
@@ -3955,16 +4320,25 @@
   <dataFields count="1">
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="2">
-    <format dxfId="92">
+  <formats count="3">
+    <format dxfId="121">
       <pivotArea field="3" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="91">
+    <format dxfId="120">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
+    <format dxfId="53">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="3" count="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
   </formats>
-  <conditionalFormats count="2">
-    <conditionalFormat priority="4">
+  <conditionalFormats count="4">
+    <conditionalFormat priority="20">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -3982,7 +4356,7 @@
         </pivotArea>
       </pivotAreas>
     </conditionalFormat>
-    <conditionalFormat priority="3">
+    <conditionalFormat priority="19">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -3995,6 +4369,34 @@
               <x v="2"/>
               <x v="3"/>
               <x v="4"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+    <conditionalFormat priority="14">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="3" count="1">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </pivotAreas>
+    </conditionalFormat>
+    <conditionalFormat priority="13">
+      <pivotAreas count="1">
+        <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+          <references count="2">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+            <reference field="3" count="1">
+              <x v="0"/>
             </reference>
           </references>
         </pivotArea>
@@ -4015,7 +4417,7 @@
 
 <file path=xl/pivotTables/pivotTable15.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FFBC07AA-ACC0-49E5-BC9B-2B10D6352CD6}" name="Tableau croisé dynamique32" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valeurs" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B20:C29" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="B23:C32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField dataField="1" showAll="0">
       <items count="16">
@@ -4101,12 +4503,25 @@
   <dataFields count="1">
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="2">
-    <format dxfId="94">
+  <formats count="3">
+    <format dxfId="54">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="93">
+    <format dxfId="55">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+    <format dxfId="56">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="5">
+            <x v="3"/>
+            <x v="4"/>
+            <x v="5"/>
+            <x v="6"/>
+            <x v="7"/>
+          </reference>
+        </references>
+      </pivotArea>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -4222,7 +4637,7 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="8">
-    <format dxfId="47">
+    <format dxfId="77">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -4234,7 +4649,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="46">
+    <format dxfId="76">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -4246,7 +4661,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="45">
+    <format dxfId="75">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -4258,7 +4673,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="44">
+    <format dxfId="74">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -4270,20 +4685,20 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="43">
+    <format dxfId="73">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="72">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="41">
+    <format dxfId="71">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="70">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="3" count="1" selected="0">
@@ -4396,7 +4811,7 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="53">
+    <format dxfId="83">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="4" selected="0">
@@ -4411,7 +4826,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="52">
+    <format dxfId="82">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="1" selected="0">
@@ -4423,7 +4838,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="51">
+    <format dxfId="81">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="2" count="1" selected="0">
@@ -4435,13 +4850,13 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="50">
+    <format dxfId="80">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="49">
+    <format dxfId="79">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="48">
+    <format dxfId="78">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -4618,29 +5033,29 @@
     <dataField name="Nombre de transaction_id" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="24">
-    <format dxfId="77">
+    <format dxfId="107">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="76">
+    <format dxfId="106">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="75">
+    <format dxfId="105">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="74">
+    <format dxfId="104">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="73">
+    <format dxfId="103">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="102">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="71">
+    <format dxfId="101">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4653,7 +5068,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="70">
+    <format dxfId="100">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4666,7 +5081,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="69">
+    <format dxfId="99">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4679,7 +5094,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="68">
+    <format dxfId="98">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4692,7 +5107,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="67">
+    <format dxfId="97">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4705,7 +5120,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="66">
+    <format dxfId="96">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4718,7 +5133,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="65">
+    <format dxfId="95">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4731,7 +5146,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="64">
+    <format dxfId="94">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4744,7 +5159,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="63">
+    <format dxfId="93">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -4757,7 +5172,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="62">
+    <format dxfId="92">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1">
@@ -4769,7 +5184,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="61">
+    <format dxfId="91">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -4778,7 +5193,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="60">
+    <format dxfId="90">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -4787,7 +5202,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="59">
+    <format dxfId="89">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="7">
@@ -4802,7 +5217,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="58">
+    <format dxfId="88">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -4811,7 +5226,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="87">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -4820,7 +5235,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="56">
+    <format dxfId="86">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -4833,7 +5248,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="55">
+    <format dxfId="85">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -4846,7 +5261,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="54">
+    <format dxfId="84">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -4941,10 +5356,10 @@
     <dataField name="CA" fld="5" baseField="6" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="79">
+    <format dxfId="109">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="78">
+    <format dxfId="108">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -5034,7 +5449,7 @@
     <dataField name="Chiffre d'affaire" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="157">
+    <format dxfId="184">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="1">
@@ -5043,7 +5458,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="156">
+    <format dxfId="183">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="1">
@@ -5166,7 +5581,7 @@
     <dataField name="Chiffre d'affaire" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="163">
+    <format dxfId="190">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -5175,7 +5590,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="162">
+    <format dxfId="189">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -5184,7 +5599,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="161">
+    <format dxfId="188">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -5193,7 +5608,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="160">
+    <format dxfId="187">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -5202,7 +5617,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="159">
+    <format dxfId="186">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -5211,7 +5626,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="158">
+    <format dxfId="185">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="3" count="1">
@@ -5419,10 +5834,10 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="113">
+    <format dxfId="140">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="112">
+    <format dxfId="139">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -5645,7 +6060,7 @@
     <dataField name="Somme de montant_fc" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="28">
-    <format dxfId="141">
+    <format dxfId="168">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="1" count="2">
@@ -5658,10 +6073,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="140">
+    <format dxfId="167">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="139">
+    <format dxfId="166">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5674,7 +6089,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="138">
+    <format dxfId="165">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5687,7 +6102,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="137">
+    <format dxfId="164">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5700,7 +6115,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="136">
+    <format dxfId="163">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5713,7 +6128,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="135">
+    <format dxfId="162">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5726,7 +6141,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="134">
+    <format dxfId="161">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5739,7 +6154,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="133">
+    <format dxfId="160">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5752,7 +6167,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="132">
+    <format dxfId="159">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="2">
@@ -5765,7 +6180,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="131">
+    <format dxfId="158">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -5774,7 +6189,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="130">
+    <format dxfId="157">
       <pivotArea field="2" dataOnly="0" labelOnly="1" grandCol="1" outline="0" axis="axisCol" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -5783,10 +6198,10 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="129">
+    <format dxfId="156">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="128">
+    <format dxfId="155">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="2" selected="0">
@@ -5803,7 +6218,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="127">
+    <format dxfId="154">
       <pivotArea dataOnly="0" labelOnly="1" offset="A256" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5812,7 +6227,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="126">
+    <format dxfId="153">
       <pivotArea dataOnly="0" labelOnly="1" offset="IV256" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5821,7 +6236,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="125">
+    <format dxfId="152">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5830,7 +6245,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="124">
+    <format dxfId="151">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5839,7 +6254,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="123">
+    <format dxfId="150">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5848,7 +6263,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="122">
+    <format dxfId="149">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5857,7 +6272,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="121">
+    <format dxfId="148">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5866,7 +6281,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="120">
+    <format dxfId="147">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5875,7 +6290,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="119">
+    <format dxfId="146">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="1">
@@ -5884,7 +6299,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="118">
+    <format dxfId="145">
       <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" axis="axisCol" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5894,7 +6309,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="117">
+    <format dxfId="144">
       <pivotArea field="2" grandRow="1" outline="0" collapsedLevelsAreSubtotals="1" axis="axisCol" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5904,7 +6319,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="116">
+    <format dxfId="143">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="2" selected="0">
@@ -5918,7 +6333,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="115">
+    <format dxfId="142">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -5931,7 +6346,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="114">
+    <format dxfId="141">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="3">
           <reference field="4294967294" count="1" selected="0">
@@ -6098,17 +6513,17 @@
     <dataField name="Canal preferé par client" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="144">
+    <format dxfId="171">
       <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="143">
+    <format dxfId="170">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="6" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="142">
+    <format dxfId="169">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -6193,10 +6608,10 @@
     <dataField name="Somme de montant_fc" fld="6" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="29">
+    <format dxfId="59">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="30">
+    <format dxfId="60">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="2">
@@ -6345,16 +6760,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6EC83A65-D9A6-475F-8D16-1CE811FFF2E9}" name="Tableau1" displayName="Tableau1" ref="B3:H13" totalsRowShown="0" headerRowDxfId="153" dataDxfId="152">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6EC83A65-D9A6-475F-8D16-1CE811FFF2E9}" name="Tableau1" displayName="Tableau1" ref="B3:H13" totalsRowShown="0" headerRowDxfId="180" dataDxfId="179">
   <autoFilter ref="B3:H13" xr:uid="{6EC83A65-D9A6-475F-8D16-1CE811FFF2E9}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{54537CD7-847D-4C04-9BD6-B993FB8C0924}" name="transaction_id" dataDxfId="151"/>
-    <tableColumn id="2" xr3:uid="{7DFAA592-DC98-463C-A6AF-A94A0F915646}" name="date" dataDxfId="150"/>
-    <tableColumn id="3" xr3:uid="{122DF7BD-714F-4B55-830F-7573F364E80A}" name="client_id" dataDxfId="149"/>
-    <tableColumn id="4" xr3:uid="{1B94713D-DD23-416E-B23B-98EF629AFCBE}" name="commune" dataDxfId="148"/>
-    <tableColumn id="5" xr3:uid="{084E48D7-3EDD-4FC4-B38B-BD3872EDFF23}" name="produit" dataDxfId="147"/>
-    <tableColumn id="6" xr3:uid="{D1BF92F6-B520-4D49-B97E-C1395DDE5A98}" name="montant_fc" dataDxfId="146"/>
-    <tableColumn id="7" xr3:uid="{21C18558-D71D-47B7-B0D0-001594508953}" name="canal" dataDxfId="145"/>
+    <tableColumn id="1" xr3:uid="{54537CD7-847D-4C04-9BD6-B993FB8C0924}" name="transaction_id" dataDxfId="178"/>
+    <tableColumn id="2" xr3:uid="{7DFAA592-DC98-463C-A6AF-A94A0F915646}" name="date" dataDxfId="177"/>
+    <tableColumn id="3" xr3:uid="{122DF7BD-714F-4B55-830F-7573F364E80A}" name="client_id" dataDxfId="176"/>
+    <tableColumn id="4" xr3:uid="{1B94713D-DD23-416E-B23B-98EF629AFCBE}" name="commune" dataDxfId="175"/>
+    <tableColumn id="5" xr3:uid="{084E48D7-3EDD-4FC4-B38B-BD3872EDFF23}" name="produit" dataDxfId="174"/>
+    <tableColumn id="6" xr3:uid="{D1BF92F6-B520-4D49-B97E-C1395DDE5A98}" name="montant_fc" dataDxfId="173"/>
+    <tableColumn id="7" xr3:uid="{21C18558-D71D-47B7-B0D0-001594508953}" name="canal" dataDxfId="172"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6364,13 +6779,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5B43BC6D-66A6-432F-982F-C406FA282078}" name="Dataset_day2__2" displayName="Dataset_day2__2" ref="B2:H17" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="B2:H17" xr:uid="{5B43BC6D-66A6-432F-982F-C406FA282078}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F0363F15-00D8-44D9-B9E8-73E1201A36E6}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="111"/>
-    <tableColumn id="2" xr3:uid="{85F76B94-3323-41EB-B99E-F9DE7DD9EF5D}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{90258075-E8BA-4181-AEBF-14DCE9CF1AC4}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="109"/>
-    <tableColumn id="4" xr3:uid="{3B088930-C813-470C-9790-11DA318C42A1}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="108"/>
-    <tableColumn id="5" xr3:uid="{E074DF00-E0E7-41D6-B91A-ABE22CB1881A}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="107"/>
+    <tableColumn id="1" xr3:uid="{F0363F15-00D8-44D9-B9E8-73E1201A36E6}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="138"/>
+    <tableColumn id="2" xr3:uid="{85F76B94-3323-41EB-B99E-F9DE7DD9EF5D}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="137"/>
+    <tableColumn id="3" xr3:uid="{90258075-E8BA-4181-AEBF-14DCE9CF1AC4}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="136"/>
+    <tableColumn id="4" xr3:uid="{3B088930-C813-470C-9790-11DA318C42A1}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="135"/>
+    <tableColumn id="5" xr3:uid="{E074DF00-E0E7-41D6-B91A-ABE22CB1881A}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="134"/>
     <tableColumn id="6" xr3:uid="{7C01ABE9-F9C0-40F6-9F95-D610FB820086}" uniqueName="6" name="montant_fc" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{30F6D1BA-4065-4D54-BF94-1BE05C99AC63}" uniqueName="7" name="canal" queryTableFieldId="7" dataDxfId="106"/>
+    <tableColumn id="7" xr3:uid="{30F6D1BA-4065-4D54-BF94-1BE05C99AC63}" uniqueName="7" name="canal" queryTableFieldId="7" dataDxfId="133"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6380,12 +6795,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A4A0DCA2-C1C4-44D4-AD45-BDA248A44995}" name="Dataset_day3" displayName="Dataset_day3" ref="B2:H17" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="B2:H17" xr:uid="{A4A0DCA2-C1C4-44D4-AD45-BDA248A44995}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{A0067E32-0369-4D8A-BDF1-C8B907B86BD0}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="100"/>
-    <tableColumn id="2" xr3:uid="{C68FAFFA-BEA0-4F94-BA99-6450F477971E}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="99"/>
-    <tableColumn id="3" xr3:uid="{CDF65428-BE02-471D-A8F7-90F1D8454251}" uniqueName="3" name="agent_id" queryTableFieldId="3" dataDxfId="98"/>
-    <tableColumn id="4" xr3:uid="{22F84FAA-57F1-425F-B37C-F8428C49E033}" uniqueName="4" name="client_id" queryTableFieldId="4" dataDxfId="97"/>
-    <tableColumn id="5" xr3:uid="{93A8CFD1-D585-478D-9AFB-02301838500E}" uniqueName="5" name="commune" queryTableFieldId="5" dataDxfId="96"/>
-    <tableColumn id="6" xr3:uid="{956E7CEA-E833-4F96-9E51-2D67194B8C61}" uniqueName="6" name="produit" queryTableFieldId="6" dataDxfId="95"/>
+    <tableColumn id="1" xr3:uid="{A0067E32-0369-4D8A-BDF1-C8B907B86BD0}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{C68FAFFA-BEA0-4F94-BA99-6450F477971E}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{CDF65428-BE02-471D-A8F7-90F1D8454251}" uniqueName="3" name="agent_id" queryTableFieldId="3" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{22F84FAA-57F1-425F-B37C-F8428C49E033}" uniqueName="4" name="client_id" queryTableFieldId="4" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{93A8CFD1-D585-478D-9AFB-02301838500E}" uniqueName="5" name="commune" queryTableFieldId="5" dataDxfId="123"/>
+    <tableColumn id="6" xr3:uid="{956E7CEA-E833-4F96-9E51-2D67194B8C61}" uniqueName="6" name="produit" queryTableFieldId="6" dataDxfId="122"/>
     <tableColumn id="7" xr3:uid="{E636C8A0-3C3C-48BE-AFE5-1B3DB129CA7E}" uniqueName="7" name="montant_fc" queryTableFieldId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6396,11 +6811,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AB24B926-8F3E-4EE6-9138-D47BB2378B02}" name="Dataset_day4" displayName="Dataset_day4" ref="B2:G17" totalsRowShown="0">
   <autoFilter ref="B2:G17" xr:uid="{AB24B926-8F3E-4EE6-9138-D47BB2378B02}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{2FA77349-5B7D-430C-A299-CA8EF8B94F8F}" name="transaction_id" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{EA88A0A8-EDC4-468E-80F4-EF0578FE9A03}" name="date" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{811F8411-B146-492E-A697-2D905854F94D}" name="client_id" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{7B37CE19-01A8-4470-8A2B-849B751FB37D}" name="commune" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{863A1A63-AC11-4715-82E2-F6EC444E5B51}" name="produit" dataDxfId="81"/>
+    <tableColumn id="1" xr3:uid="{2FA77349-5B7D-430C-A299-CA8EF8B94F8F}" name="transaction_id" dataDxfId="115"/>
+    <tableColumn id="2" xr3:uid="{EA88A0A8-EDC4-468E-80F4-EF0578FE9A03}" name="date" dataDxfId="114"/>
+    <tableColumn id="3" xr3:uid="{811F8411-B146-492E-A697-2D905854F94D}" name="client_id" dataDxfId="113"/>
+    <tableColumn id="4" xr3:uid="{7B37CE19-01A8-4470-8A2B-849B751FB37D}" name="commune" dataDxfId="112"/>
+    <tableColumn id="5" xr3:uid="{863A1A63-AC11-4715-82E2-F6EC444E5B51}" name="produit" dataDxfId="111"/>
     <tableColumn id="6" xr3:uid="{DDFB738A-4C05-4F97-882D-16FE65EF8A7E}" name="montant_fc"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6408,7 +6823,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B1C5B688-9C67-4CAD-9DAE-7207D5E5E850}" name="Tableau9" displayName="Tableau9" ref="AA3:AA11" totalsRowShown="0" headerRowDxfId="80">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{B1C5B688-9C67-4CAD-9DAE-7207D5E5E850}" name="Tableau9" displayName="Tableau9" ref="AA3:AA11" totalsRowShown="0" headerRowDxfId="110">
   <autoFilter ref="AA3:AA11" xr:uid="{B1C5B688-9C67-4CAD-9DAE-7207D5E5E850}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="AA4:AA11">
     <sortCondition ref="AA3:AA11"/>
@@ -6423,16 +6838,16 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C4A92EC0-501A-4751-9A16-2163E0BD39EA}" name="Dataset_day5" displayName="Dataset_day5" ref="B2:H17" tableType="queryTable" totalsRowShown="0" headerRowDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{C4A92EC0-501A-4751-9A16-2163E0BD39EA}" name="Dataset_day5" displayName="Dataset_day5" ref="B2:H17" tableType="queryTable" totalsRowShown="0" headerRowDxfId="69">
   <autoFilter ref="B2:H17" xr:uid="{C4A92EC0-501A-4751-9A16-2163E0BD39EA}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{FBC21564-1B48-423F-AFDB-04B5AE20CF75}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{CA4A50D7-5720-4F71-ACD1-3781681C0231}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{A265E5F8-50A6-4DD3-8C5E-10BB05E3F126}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{0E595B89-2727-474B-B4A6-66BC0AC0864A}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{4D992877-9744-466D-982E-E1F06CDEF762}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{FBC21564-1B48-423F-AFDB-04B5AE20CF75}" uniqueName="1" name="transaction_id" queryTableFieldId="1" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{CA4A50D7-5720-4F71-ACD1-3781681C0231}" uniqueName="2" name="date" queryTableFieldId="2" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{A265E5F8-50A6-4DD3-8C5E-10BB05E3F126}" uniqueName="3" name="client_id" queryTableFieldId="3" dataDxfId="66"/>
+    <tableColumn id="4" xr3:uid="{0E595B89-2727-474B-B4A6-66BC0AC0864A}" uniqueName="4" name="commune" queryTableFieldId="4" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{4D992877-9744-466D-982E-E1F06CDEF762}" uniqueName="5" name="produit" queryTableFieldId="5" dataDxfId="64"/>
     <tableColumn id="6" xr3:uid="{D10FAE6E-7969-4551-94AB-82C2D27DFD50}" uniqueName="6" name="montant_fc" queryTableFieldId="6"/>
-    <tableColumn id="7" xr3:uid="{7306D68B-3C9A-40F7-A0D9-E00CC8C73541}" uniqueName="7" name="periode" queryTableFieldId="7" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{7306D68B-3C9A-40F7-A0D9-E00CC8C73541}" uniqueName="7" name="periode" queryTableFieldId="7" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6443,7 +6858,7 @@
   <autoFilter ref="A1:G6" xr:uid="{68E59C74-D329-4B48-A967-CC868365949C}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C102BD58-3DF8-48B7-9114-2067608D3DB4}" name="transaction_id"/>
-    <tableColumn id="2" xr3:uid="{998F6E83-476D-414D-8353-8E6146354739}" name="date" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{998F6E83-476D-414D-8353-8E6146354739}" name="date" dataDxfId="62"/>
     <tableColumn id="3" xr3:uid="{1ACC5CD9-2A0F-4DB2-B7B7-A25781DA1795}" name="agent_id"/>
     <tableColumn id="4" xr3:uid="{D4B111D2-01DE-4AFC-91B0-641E23172B8C}" name="client_id"/>
     <tableColumn id="5" xr3:uid="{C0E2906A-2633-4FB3-89D8-883ADDF86D4F}" name="commune"/>
@@ -7163,24 +7578,24 @@
       </c>
     </row>
     <row r="26" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="59" t="s">
+      <c r="B26" s="60" t="s">
         <v>205</v>
       </c>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
     </row>
     <row r="27" spans="2:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="59"/>
-      <c r="C27" s="59"/>
-      <c r="D27" s="59"/>
+      <c r="B27" s="60"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="60"/>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
+      <c r="B28" s="61"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="61"/>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B29" s="58"/>
+      <c r="B29" s="59"/>
       <c r="C29" s="10"/>
     </row>
     <row r="30" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7256,12 +7671,12 @@
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="58" t="s">
+      <c r="B41" s="59" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B42" s="58"/>
+      <c r="B42" s="59"/>
     </row>
     <row r="44" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B44" s="50" t="s">
@@ -7329,13 +7744,13 @@
       <c r="C53" s="10"/>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B54" s="58" t="s">
+      <c r="B54" s="59" t="s">
         <v>208</v>
       </c>
       <c r="C54" s="10"/>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B55" s="58"/>
+      <c r="B55" s="59"/>
       <c r="C55" s="10"/>
     </row>
     <row r="57" spans="2:4" ht="18.75" x14ac:dyDescent="0.25">
@@ -8039,13 +8454,13 @@
       <c r="C34" s="10"/>
     </row>
     <row r="35" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="58" t="s">
+      <c r="B35" s="59" t="s">
         <v>201</v>
       </c>
       <c r="C35" s="10"/>
     </row>
     <row r="36" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="58"/>
+      <c r="B36" s="59"/>
       <c r="C36" s="10"/>
     </row>
     <row r="37" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -8587,12 +9002,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="C80:C81">
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="3" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="C80:C81">
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9025,12 +9440,12 @@
       </c>
     </row>
     <row r="20" spans="2:8" s="19" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="56" t="s">
+      <c r="B20" s="57" t="s">
         <v>193</v>
       </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="56"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="48" t="s">
@@ -9127,12 +9542,12 @@
       </c>
     </row>
     <row r="33" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="56" t="s">
+      <c r="B33" s="57" t="s">
         <v>194</v>
       </c>
-      <c r="C33" s="56"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="56"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="57"/>
+      <c r="E33" s="57"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" s="48" t="s">
@@ -9229,12 +9644,12 @@
       </c>
     </row>
     <row r="46" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="56" t="s">
+      <c r="B46" s="57" t="s">
         <v>196</v>
       </c>
-      <c r="C46" s="56"/>
-      <c r="D46" s="56"/>
-      <c r="E46" s="56"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="57"/>
+      <c r="E46" s="57"/>
     </row>
     <row r="47" spans="2:8" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B47" s="42"/>
@@ -9372,33 +9787,33 @@
       </c>
     </row>
     <row r="57" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B57" s="57" t="s">
+      <c r="B57" s="58" t="s">
         <v>200</v>
       </c>
-      <c r="C57" s="57"/>
-      <c r="D57" s="57"/>
-      <c r="E57" s="57"/>
-      <c r="F57" s="57"/>
-      <c r="G57" s="57"/>
-      <c r="H57" s="57"/>
+      <c r="C57" s="58"/>
+      <c r="D57" s="58"/>
+      <c r="E57" s="58"/>
+      <c r="F57" s="58"/>
+      <c r="G57" s="58"/>
+      <c r="H57" s="58"/>
     </row>
     <row r="58" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B58" s="57"/>
-      <c r="C58" s="57"/>
-      <c r="D58" s="57"/>
-      <c r="E58" s="57"/>
-      <c r="F58" s="57"/>
-      <c r="G58" s="57"/>
-      <c r="H58" s="57"/>
+      <c r="B58" s="58"/>
+      <c r="C58" s="58"/>
+      <c r="D58" s="58"/>
+      <c r="E58" s="58"/>
+      <c r="F58" s="58"/>
+      <c r="G58" s="58"/>
+      <c r="H58" s="58"/>
     </row>
     <row r="59" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B59" s="57"/>
-      <c r="C59" s="57"/>
-      <c r="D59" s="57"/>
-      <c r="E59" s="57"/>
-      <c r="F59" s="57"/>
-      <c r="G59" s="57"/>
-      <c r="H59" s="57"/>
+      <c r="B59" s="58"/>
+      <c r="C59" s="58"/>
+      <c r="D59" s="58"/>
+      <c r="E59" s="58"/>
+      <c r="F59" s="58"/>
+      <c r="G59" s="58"/>
+      <c r="H59" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -9413,7 +9828,7 @@
     <mergeCell ref="B33:E33"/>
   </mergeCells>
   <conditionalFormatting pivot="1" sqref="D24:D28">
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="11" operator="lessThan">
       <formula>10000</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9430,7 +9845,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24:B28">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="21" priority="5" operator="lessThan">
       <formula>10000</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9447,12 +9862,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="D37:D41">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="3" operator="lessThan">
       <formula>$Q$4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting pivot="1" sqref="D37:D42">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>30000</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9477,13 +9892,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84601EC8-C861-4E54-B5F8-83B9BDC7AB04}">
-  <dimension ref="B2:AA29"/>
+  <dimension ref="B1:AA72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
     <col min="2" max="2" width="15.5703125" customWidth="1"/>
     <col min="3" max="3" width="14.140625" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
     <col min="6" max="6" width="14.42578125" customWidth="1"/>
     <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -9506,6 +9921,16 @@
     <col min="29" max="29" width="7.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="2:27" x14ac:dyDescent="0.25">
+      <c r="B1" s="48" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+    </row>
     <row r="2" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
@@ -10147,7 +10572,7 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="10" t="s">
         <v>133</v>
       </c>
@@ -10167,189 +10592,472 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="20" spans="2:10" s="19" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="20" t="s">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F18" s="10"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F19" s="10"/>
+    </row>
+    <row r="20" spans="2:7" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B20" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="10"/>
+    </row>
+    <row r="21" spans="2:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="10"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="48" t="s">
+        <v>211</v>
+      </c>
+      <c r="C22" s="48"/>
+      <c r="D22" s="65"/>
+      <c r="F22" s="10"/>
+    </row>
+    <row r="23" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B23" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C23" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="D23" s="10"/>
+      <c r="G23" s="19"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" s="10">
+        <v>5</v>
+      </c>
+      <c r="D24" s="10"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="10">
+        <v>3</v>
+      </c>
+      <c r="D25" s="10"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="C26" s="10">
+        <v>2</v>
+      </c>
+      <c r="D26" s="10"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C27" s="63">
+        <v>1</v>
+      </c>
+      <c r="D27" s="10"/>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="C28" s="63">
+        <v>1</v>
+      </c>
+      <c r="D28" s="10"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="63">
+        <v>1</v>
+      </c>
+      <c r="D29" s="10"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="C30" s="63">
+        <v>1</v>
+      </c>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="C31" s="63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="J33"/>
+    </row>
+    <row r="34" spans="2:10" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="62" t="s">
+        <v>212</v>
+      </c>
+      <c r="C34" s="62"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="62"/>
+      <c r="J34"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" s="62"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="62"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B36" s="64"/>
+      <c r="C36" s="64"/>
+      <c r="D36" s="64"/>
+      <c r="E36" s="64"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B37" s="64"/>
+      <c r="C37" s="64"/>
+      <c r="D37" s="64"/>
+      <c r="E37" s="64"/>
+    </row>
+    <row r="38" spans="2:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="B38" s="57" t="s">
+        <v>213</v>
+      </c>
+      <c r="C38" s="57"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="57"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="C40" s="48"/>
+      <c r="D40" s="65"/>
+    </row>
+    <row r="41" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="B41" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="C41" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="H20" s="20" t="s">
+      <c r="D41" s="66" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B42" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="10">
+        <v>6</v>
+      </c>
+      <c r="D42" s="67">
+        <f>C42/GETPIVOTDATA("transaction_id",$B$41)</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B43" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" s="10">
+        <v>3</v>
+      </c>
+      <c r="D43" s="67">
+        <f t="shared" ref="D43:D47" si="1">C43/GETPIVOTDATA("transaction_id",$B$41)</f>
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B44" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C44" s="10">
+        <v>2</v>
+      </c>
+      <c r="D44" s="67">
+        <f t="shared" si="1"/>
+        <v>0.13333333333333333</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B45" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" s="10">
+        <v>2</v>
+      </c>
+      <c r="D45" s="67">
+        <f t="shared" si="1"/>
+        <v>0.13333333333333333</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B46" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C46" s="10">
+        <v>2</v>
+      </c>
+      <c r="D46" s="67">
+        <f t="shared" si="1"/>
+        <v>0.13333333333333333</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B47" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C47" s="10">
+        <v>15</v>
+      </c>
+      <c r="D47" s="68">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B49" s="62" t="s">
+        <v>220</v>
+      </c>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50" s="62"/>
+      <c r="C50" s="62"/>
+      <c r="D50" s="62"/>
+      <c r="E50" s="62"/>
+    </row>
+    <row r="52" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="C52" s="56"/>
+      <c r="D52" s="56"/>
+      <c r="E52" s="56"/>
+    </row>
+    <row r="53" spans="2:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="56"/>
+      <c r="C53" s="56"/>
+      <c r="D53" s="56"/>
+      <c r="E53" s="56"/>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B55" s="48" t="s">
+        <v>217</v>
+      </c>
+      <c r="C55" s="48"/>
+      <c r="D55" s="65"/>
+    </row>
+    <row r="56" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B56" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="I20" s="19" t="s">
+      <c r="C56" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="J20"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21" s="10">
-        <v>5</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" s="10">
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B57" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C57" s="10">
         <v>6</v>
       </c>
-      <c r="H21" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I21" s="23">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B22" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="C22" s="10">
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B58" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="10">
         <v>3</v>
       </c>
-      <c r="E22" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" s="10">
-        <v>3</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="I22" s="10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B23" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="C23" s="10">
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B59" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C59" s="10">
         <v>2</v>
       </c>
-      <c r="E23" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="F23" s="10">
-        <v>2</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" s="10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B24" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="C24" s="10">
-        <v>1</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="10">
-        <v>2</v>
-      </c>
-      <c r="H24" s="9" t="s">
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B60" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I24" s="10">
+      <c r="C60" s="10">
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="C25" s="10">
-        <v>1</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F25" s="10">
-        <v>2</v>
-      </c>
-      <c r="H25" s="9" t="s">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B61" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I25" s="10">
+      <c r="C61" s="10">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B26" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C26" s="10">
-        <v>1</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F26" s="10">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="C27" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B28" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="C28" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C29" s="10">
-        <v>15</v>
-      </c>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B63" s="62" t="s">
+        <v>218</v>
+      </c>
+      <c r="C63" s="62"/>
+      <c r="D63" s="62"/>
+      <c r="E63" s="62"/>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B64" s="62"/>
+      <c r="C64" s="62"/>
+      <c r="D64" s="62"/>
+      <c r="E64" s="62"/>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B65" s="64"/>
+      <c r="C65" s="64"/>
+      <c r="D65" s="64"/>
+      <c r="E65" s="64"/>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B66" s="64"/>
+      <c r="C66" s="64"/>
+      <c r="D66" s="64"/>
+      <c r="E66" s="64"/>
+    </row>
+    <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B67" s="62" t="s">
+        <v>219</v>
+      </c>
+      <c r="C67" s="62"/>
+      <c r="D67" s="62"/>
+      <c r="E67" s="62"/>
+      <c r="F67" s="62"/>
+    </row>
+    <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B68" s="62"/>
+      <c r="C68" s="62"/>
+      <c r="D68" s="62"/>
+      <c r="E68" s="62"/>
+      <c r="F68" s="62"/>
+    </row>
+    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B69" s="62"/>
+      <c r="C69" s="62"/>
+      <c r="D69" s="62"/>
+      <c r="E69" s="62"/>
+      <c r="F69" s="62"/>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B70" s="62"/>
+      <c r="C70" s="62"/>
+      <c r="D70" s="62"/>
+      <c r="E70" s="62"/>
+      <c r="F70" s="62"/>
+    </row>
+    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B71" s="62"/>
+      <c r="C71" s="62"/>
+      <c r="D71" s="62"/>
+      <c r="E71" s="62"/>
+      <c r="F71" s="62"/>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B72" s="62"/>
+      <c r="C72" s="62"/>
+      <c r="D72" s="62"/>
+      <c r="E72" s="62"/>
+      <c r="F72" s="62"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B20:C29">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
+  <mergeCells count="11">
+    <mergeCell ref="B49:E50"/>
+    <mergeCell ref="B63:E64"/>
+    <mergeCell ref="B67:F72"/>
+    <mergeCell ref="B34:E35"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B52:E53"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B38:E38"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B23:C32">
+    <cfRule type="cellIs" dxfId="18" priority="21" operator="lessThan">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting pivot="1" sqref="F21:F25">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
+  <conditionalFormatting pivot="1" sqref="C42:C46">
+    <cfRule type="cellIs" dxfId="17" priority="20" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting pivot="1" sqref="F21:F25">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+  <conditionalFormatting pivot="1" sqref="C42:C46">
+    <cfRule type="cellIs" dxfId="16" priority="19" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA4:AA11">
-    <cfRule type="top10" dxfId="1" priority="1" rank="2"/>
-    <cfRule type="top10" dxfId="0" priority="2" rank="2"/>
+    <cfRule type="top10" dxfId="15" priority="17" rank="2"/>
+    <cfRule type="top10" dxfId="14" priority="18" rank="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting pivot="1" sqref="C42">
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="greaterThan">
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting pivot="1" sqref="C42">
+    <cfRule type="cellIs" dxfId="12" priority="13" operator="greaterThan">
+      <formula>3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting pivot="1" sqref="C57">
+    <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">
+      <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting pivot="1" sqref="C57">
+    <cfRule type="cellIs" dxfId="10" priority="11" operator="greaterThan">
+      <formula>5</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting pivot="1" sqref="C57">
+    <cfRule type="cellIs" dxfId="9" priority="10" operator="greaterThan">
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting pivot="1" sqref="C57">
+    <cfRule type="cellIs" dxfId="8" priority="9" operator="greaterThan">
+      <formula>3</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
   <tableParts count="2">
-    <tablePart r:id="rId5"/>
     <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>